<commit_message>
Adding applications V7.00 AI SDK
</commit_message>
<xml_diff>
--- a/06_Face_recognition_spoof_detection/Face_spoof_detection_img/exe/resnet50_classifier_bmp/resnet50_classifier_bmp_summary.xlsx
+++ b/06_Face_recognition_spoof_detection/Face_spoof_detection_img/exe/resnet50_classifier_bmp/resnet50_classifier_bmp_summary.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>/conv1/Conv_output_0</t>
+          <t>496</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/maxpool/MaxPool_output_0</t>
+          <t>324</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/layer1/layer1.0/conv1/Conv_output_0</t>
+          <t>499</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/layer1/layer1.0/conv2/Conv_output_0</t>
+          <t>502</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/layer1/layer1.0/conv3/Conv_output_0</t>
+          <t>505</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/layer1/layer1.0/downsample/downsample.0/Conv_output_0</t>
+          <t>508</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/layer1/layer1.0/Add_output_0</t>
+          <t>335</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/layer1/layer1.1/conv1/Conv_output_0</t>
+          <t>511</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/layer1/layer1.1/conv2/Conv_output_0</t>
+          <t>514</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/layer1/layer1.1/conv3/Conv_output_0</t>
+          <t>517</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/layer1/layer1.1/Add_output_0</t>
+          <t>345</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/layer1/layer1.2/conv1/Conv_output_0</t>
+          <t>520</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/layer1/layer1.2/conv2/Conv_output_0</t>
+          <t>523</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/layer1/layer1.2/conv3/Conv_output_0</t>
+          <t>526</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/layer1/layer1.2/Add_output_0</t>
+          <t>355</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/layer2/layer2.0/conv1/Conv_output_0</t>
+          <t>529</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/layer2/layer2.0/conv2/Conv_output_0</t>
+          <t>532</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/layer2/layer2.0/conv3/Conv_output_0</t>
+          <t>535</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/layer2/layer2.0/downsample/downsample.0/Conv_output_0</t>
+          <t>538</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/layer2/layer2.0/Add_output_0</t>
+          <t>367</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/layer2/layer2.1/conv1/Conv_output_0</t>
+          <t>541</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/layer2/layer2.1/conv2/Conv_output_0</t>
+          <t>544</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/layer2/layer2.1/conv3/Conv_output_0</t>
+          <t>547</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/layer2/layer2.1/Add_output_0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/layer2/layer2.2/conv1/Conv_output_0</t>
+          <t>550</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/layer2/layer2.2/conv2/Conv_output_0</t>
+          <t>553</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/layer2/layer2.2/conv3/Conv_output_0</t>
+          <t>556</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/layer2/layer2.2/Add_output_0</t>
+          <t>387</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/layer2/layer2.3/conv1/Conv_output_0</t>
+          <t>559</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/layer2/layer2.3/conv2/Conv_output_0</t>
+          <t>562</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/layer2/layer2.3/conv3/Conv_output_0</t>
+          <t>565</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/layer2/layer2.3/Add_output_0</t>
+          <t>397</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/layer3/layer3.0/conv1/Conv_output_0</t>
+          <t>568</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/layer3/layer3.0/conv2/Conv_output_0</t>
+          <t>571</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/layer3/layer3.0/conv3/Conv_output_0</t>
+          <t>574</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/layer3/layer3.0/downsample/downsample.0/Conv_output_0</t>
+          <t>577</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/layer3/layer3.0/Add_output_0</t>
+          <t>409</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/layer3/layer3.1/conv1/Conv_output_0</t>
+          <t>580</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/layer3/layer3.1/conv2/Conv_output_0</t>
+          <t>583</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/layer3/layer3.1/conv3/Conv_output_0</t>
+          <t>586</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/layer3/layer3.1/Add_output_0</t>
+          <t>419</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/layer3/layer3.2/conv1/Conv_output_0</t>
+          <t>589</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/layer3/layer3.2/conv2/Conv_output_0</t>
+          <t>592</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/layer3/layer3.2/conv3/Conv_output_0</t>
+          <t>595</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/layer3/layer3.2/Add_output_0</t>
+          <t>429</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/layer3/layer3.3/conv1/Conv_output_0</t>
+          <t>598</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>/layer3/layer3.3/conv2/Conv_output_0</t>
+          <t>601</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/layer3/layer3.3/conv3/Conv_output_0</t>
+          <t>604</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/layer3/layer3.3/Add_output_0</t>
+          <t>439</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/layer3/layer3.4/conv1/Conv_output_0</t>
+          <t>607</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>/layer3/layer3.4/conv2/Conv_output_0</t>
+          <t>610</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/layer3/layer3.4/conv3/Conv_output_0</t>
+          <t>613</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/layer3/layer3.4/Add_output_0</t>
+          <t>449</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>/layer3/layer3.5/conv1/Conv_output_0</t>
+          <t>616</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>/layer3/layer3.5/conv2/Conv_output_0</t>
+          <t>619</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>/layer3/layer3.5/conv3/Conv_output_0</t>
+          <t>622</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>/layer3/layer3.5/Add_output_0</t>
+          <t>459</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>/layer4/layer4.0/conv1/Conv_output_0</t>
+          <t>625</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>/layer4/layer4.0/conv2/Conv_output_0</t>
+          <t>628</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>/layer4/layer4.0/conv3/Conv_output_0</t>
+          <t>631</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>/layer4/layer4.0/downsample/downsample.0/Conv_output_0</t>
+          <t>634</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>/layer4/layer4.0/Add_output_0</t>
+          <t>471</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>/layer4/layer4.1/conv1/Conv_output_0</t>
+          <t>637</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>/layer4/layer4.1/conv2/Conv_output_0</t>
+          <t>640</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>/layer4/layer4.1/conv3/Conv_output_0</t>
+          <t>643</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>/layer4/layer4.1/Add_output_0</t>
+          <t>481</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -4738,7 +4738,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>/layer4/layer4.2/conv1/Conv_output_0</t>
+          <t>646</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>/layer4/layer4.2/conv2/Conv_output_0</t>
+          <t>649</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>/layer4/layer4.2/conv3/Conv_output_0</t>
+          <t>652</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>/layer4/layer4.2/Add_output_0</t>
+          <t>491</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>/avgpool/GlobalAveragePool_output_0</t>
+          <t>493</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">

</xml_diff>